<commit_message>
Latest data: Mon Apr 20 13:12:07 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -667,11 +667,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3697</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>9</v>
+        <v>258</v>
       </c>
     </row>
     <row r="20">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>324337</t>
+          <t>2068/43</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>258</v>
+        <v>310</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>655248</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>258</v>
+        <v>310</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>258</v>
+        <v>310</v>
       </c>
     </row>
     <row r="23">
@@ -719,7 +719,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>310</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>4052</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>310</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>310</v>
+        <v>140</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4052</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>2727/1</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>140</v>
+        <v>189</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>47/3</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>140</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>302/1</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>187</v>
+        <v>277</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>2103/7</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>189</v>
+        <v>394</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>673/2</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>277</v>
+        <v>384</v>
       </c>
     </row>
     <row r="34">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>.372</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>277</v>
+        <v>384</v>
       </c>
     </row>
     <row r="35">
@@ -875,11 +875,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>.373</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>394</v>
+        <v>384</v>
       </c>
     </row>
     <row r="36">
@@ -888,7 +888,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>673/2</t>
+          <t>.374</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -901,7 +901,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>.372</t>
+          <t>673/2</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>.373</t>
+          <t>406/3</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -927,7 +927,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>.374</t>
+          <t>605</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -940,7 +940,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>673/2</t>
+          <t>657/1</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -953,7 +953,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>406/3</t>
+          <t>674</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>605</t>
+          <t>765/3</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -979,7 +979,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>657/1</t>
+          <t>938</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -992,7 +992,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>674</t>
+          <t>996</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>765/3</t>
+          <t>2074</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>938</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>996</t>
+          <t>2065</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2074</t>
+          <t>2066</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2153</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2065</t>
+          <t>2154</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1083,11 +1083,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2066</t>
+          <t>1419</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>384</v>
+        <v>287</v>
       </c>
     </row>
     <row r="52">
@@ -1096,11 +1096,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2153</t>
+          <t>1420</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>384</v>
+        <v>287</v>
       </c>
     </row>
     <row r="53">
@@ -1109,11 +1109,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2154</t>
+          <t>1421</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>384</v>
+        <v>287</v>
       </c>
     </row>
     <row r="54">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1419</t>
+          <t>1430</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>1431/1</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1421</t>
+          <t>1431/34</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1430</t>
+          <t>.950/1</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1431/1</t>
+          <t>.950/2</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1431/34</t>
+          <t>239</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>.950/1</t>
+          <t>241</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -1213,11 +1213,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>.950/2</t>
+          <t>773</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>287</v>
+        <v>441</v>
       </c>
     </row>
     <row r="62">
@@ -1226,11 +1226,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>.798</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>287</v>
+        <v>307</v>
       </c>
     </row>
     <row r="63">
@@ -1239,11 +1239,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>.4046</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>287</v>
+        <v>307</v>
       </c>
     </row>
     <row r="64">
@@ -1252,11 +1252,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>773</t>
+          <t>.4047</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>441</v>
+        <v>307</v>
       </c>
     </row>
     <row r="65">
@@ -1265,11 +1265,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>.798</t>
+          <t>1133</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>307</v>
+        <v>248</v>
       </c>
     </row>
     <row r="66">
@@ -1278,11 +1278,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>1585/60</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>307</v>
+        <v>248</v>
       </c>
     </row>
     <row r="67">
@@ -1291,49 +1291,10 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>.4047</t>
+          <t>1064/3</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>66</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>1133</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>67</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1585/60</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="n">
-        <v>68</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1064/3</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Thu Apr 30 13:25:08 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -680,7 +680,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -693,7 +693,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>310</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>4052</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>139</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4052</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26">
@@ -758,7 +758,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>140</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>2727/1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>47/3</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>189</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30">
@@ -810,7 +810,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>302/1</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>2103/7</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>277</v>
+        <v>394</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>673/2</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>394</v>
+        <v>384</v>
       </c>
     </row>
     <row r="33">
@@ -849,7 +849,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>673/2</t>
+          <t>.372</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -862,7 +862,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>.372</t>
+          <t>.373</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -875,7 +875,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>.373</t>
+          <t>.374</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -888,7 +888,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>.374</t>
+          <t>673/2</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -901,7 +901,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>673/2</t>
+          <t>406/3</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>406/3</t>
+          <t>605</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -927,7 +927,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>605</t>
+          <t>657/1</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -940,7 +940,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>657/1</t>
+          <t>674</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -953,7 +953,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>674</t>
+          <t>765/3</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>765/3</t>
+          <t>938</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -979,7 +979,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>938</t>
+          <t>996</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -992,7 +992,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>996</t>
+          <t>2074</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2074</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2065</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2065</t>
+          <t>2066</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2066</t>
+          <t>2153</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2153</t>
+          <t>2154</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1070,11 +1070,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2154</t>
+          <t>1419</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>384</v>
+        <v>287</v>
       </c>
     </row>
     <row r="51">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1419</t>
+          <t>1420</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>1421</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1421</t>
+          <t>1430</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1430</t>
+          <t>1431/1</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1431/1</t>
+          <t>1431/34</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>1431/34</t>
+          <t>.950/1</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>.950/1</t>
+          <t>.950/2</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>.950/2</t>
+          <t>239</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>241</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -1200,11 +1200,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>241</t>
+          <t>773</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>287</v>
+        <v>441</v>
       </c>
     </row>
     <row r="61">
@@ -1213,11 +1213,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>773</t>
+          <t>.798</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>441</v>
+        <v>307</v>
       </c>
     </row>
     <row r="62">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>.798</t>
+          <t>.4046</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>.4047</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -1252,49 +1252,10 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>.4047</t>
+          <t>1064/3</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>63</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>1133</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>64</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>1585/60</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>65</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>1064/3</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Thu Apr 30 17:16:13 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4052</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25">
@@ -745,7 +745,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>140</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>2727/1</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>47/3</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>189</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29">
@@ -797,7 +797,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>302/1</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>2103/7</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>277</v>
+        <v>394</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>.798</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>394</v>
+        <v>307</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>673/2</t>
+          <t>.4046</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>384</v>
+        <v>307</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.372</t>
+          <t>.4047</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>384</v>
+        <v>307</v>
       </c>
     </row>
     <row r="34">
@@ -862,400 +862,10 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>.373</t>
+          <t>1064/3</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>33</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>.374</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>673/2</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>406/3</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>605</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>657/1</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>674</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>765/3</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>938</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>996</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>2074</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2050</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>2065</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2066</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>2153</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>2154</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>1419</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>1420</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>1421</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>1430</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>1431/1</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>1431/34</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>.950/1</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>.950/2</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>239</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>241</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>58</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>773</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>59</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>.798</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>60</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>.4046</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>61</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>.4047</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>62</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>1064/3</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Wed May  6 10:17:26 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -667,7 +667,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>324337</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>655248</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>310</v>
+        <v>258</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>310</v>
+        <v>258</v>
       </c>
     </row>
     <row r="22">
@@ -706,7 +706,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>139</v>
+        <v>310</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>140</v>
+        <v>310</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>187</v>
+        <v>140</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>189</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>277</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>2727/1</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>277</v>
+        <v>189</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>47/3</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>394</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>.798</t>
+          <t>302/1</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>307</v>
+        <v>277</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>2103/7</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>307</v>
+        <v>394</v>
       </c>
     </row>
     <row r="33">
@@ -849,7 +849,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.4047</t>
+          <t>.798</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -862,10 +862,36 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>.4046</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>.4047</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>1064/3</t>
         </is>
       </c>
-      <c r="C34" t="n">
+      <c r="C36" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Wed May  6 13:33:30 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,7 +615,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3053</t>
+          <t>3597/16</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -628,7 +628,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3597/16</t>
+          <t>3597/18</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3597/18</t>
+          <t>3597/22</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -654,7 +654,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3597/22</t>
+          <t>3697</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -667,7 +667,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>324337</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>655248</t>
+          <t>2068/43</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>258</v>
+        <v>310</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>258</v>
+        <v>310</v>
       </c>
     </row>
     <row r="22">
@@ -706,7 +706,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -719,7 +719,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>310</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26">
@@ -758,7 +758,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>140</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>2727/1</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>47/3</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>189</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30">
@@ -810,7 +810,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>302/1</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>2103/7</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>277</v>
+        <v>394</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>.4047</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>394</v>
+        <v>307</v>
       </c>
     </row>
     <row r="33">
@@ -849,7 +849,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.798</t>
+          <t>.4046</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -862,36 +862,10 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>1064/3</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>33</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>.4047</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>1064/3</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Fri Jul  3 21:39:21 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,11 +563,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4523</t>
+          <t>4119</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>404</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12">
@@ -576,11 +576,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>.451</t>
+          <t>4120</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>88</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13">
@@ -589,11 +589,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>446</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>202</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14">
@@ -602,11 +602,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>4523</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>61</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15">
@@ -615,11 +615,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3597/16</t>
+          <t>2548/13</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>444</v>
       </c>
     </row>
     <row r="16">
@@ -628,11 +628,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3597/18</t>
+          <t>1115</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -641,11 +641,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3597/22</t>
+          <t>.451</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18">
@@ -654,11 +654,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3697</t>
+          <t>274</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>202</v>
       </c>
     </row>
     <row r="19">
@@ -667,11 +667,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>1341</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>258</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>703</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>310</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>3597/16</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>310</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>3597/18</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>310</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>3597/22</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>310</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>3697</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>139</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>140</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>2068/43</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>140</v>
+        <v>310</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>187</v>
+        <v>310</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>189</v>
+        <v>310</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>277</v>
+        <v>310</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>277</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>394</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>.4047</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>307</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>307</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34">
@@ -862,10 +862,88 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>2727/1</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>47/3</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>302/1</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2103/7</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>.4047</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>.4046</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>1064/3</t>
         </is>
       </c>
-      <c r="C34" t="n">
+      <c r="C40" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Sun Sep  6 15:00:54 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,11 +446,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9783/231</t>
+          <t>506</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>44</v>
+        <v>313</v>
       </c>
     </row>
     <row r="3">
@@ -459,11 +459,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>13823</t>
+          <t>824</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>154</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4">
@@ -472,11 +472,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14724/2</t>
+          <t>888</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>154</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5">
@@ -485,11 +485,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>8974/1</t>
+          <t>889</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>154</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6">
@@ -498,11 +498,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>15380</t>
+          <t>890</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>154</v>
+        <v>313</v>
       </c>
     </row>
     <row r="7">
@@ -511,11 +511,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>583</t>
+          <t>891</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>174</v>
+        <v>313</v>
       </c>
     </row>
     <row r="8">
@@ -524,11 +524,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>466</t>
+          <t>897</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>213</v>
+        <v>313</v>
       </c>
     </row>
     <row r="9">
@@ -537,11 +537,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>.315</t>
+          <t>898</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>282</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10">
@@ -550,11 +550,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>3298</t>
+          <t>899</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>257</v>
+        <v>313</v>
       </c>
     </row>
     <row r="11">
@@ -563,11 +563,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4119</t>
+          <t>900</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>256</v>
+        <v>313</v>
       </c>
     </row>
     <row r="12">
@@ -576,11 +576,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4120</t>
+          <t>901</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>256</v>
+        <v>313</v>
       </c>
     </row>
     <row r="13">
@@ -589,11 +589,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>446</t>
+          <t>9783/231</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>193</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -602,11 +602,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4523</t>
+          <t>13823</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>404</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15">
@@ -615,11 +615,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2548/13</t>
+          <t>14724/2</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>444</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16">
@@ -628,11 +628,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1115</t>
+          <t>8974/1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17">
@@ -641,11 +641,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>.451</t>
+          <t>15380</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>88</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18">
@@ -654,11 +654,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>583</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>202</v>
+        <v>174</v>
       </c>
     </row>
     <row r="19">
@@ -667,11 +667,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1341</t>
+          <t>466</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>132</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>.315</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>61</v>
+        <v>282</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3597/16</t>
+          <t>3298</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>257</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3597/18</t>
+          <t>4119</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3597/22</t>
+          <t>4120</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>256</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3697</t>
+          <t>446</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>193</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>4523</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>258</v>
+        <v>404</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>2548/13</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>310</v>
+        <v>444</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>1115</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>310</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>.451</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>310</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>274</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>310</v>
+        <v>202</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>.384</t>
+          <t>1341</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>703</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>140</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>.1512</t>
+          <t>3597/16</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>140</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.7.</t>
+          <t>3597/18</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>187</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2727/1</t>
+          <t>3597/22</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>189</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35">
@@ -875,11 +875,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>47/3</t>
+          <t>3697</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>277</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36">
@@ -888,11 +888,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>302/1</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>277</v>
+        <v>258</v>
       </c>
     </row>
     <row r="37">
@@ -901,11 +901,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2103/7</t>
+          <t>2068/43</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>394</v>
+        <v>310</v>
       </c>
     </row>
     <row r="38">
@@ -914,11 +914,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>.4047</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="39">
@@ -927,11 +927,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>.4046</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="40">
@@ -940,10 +940,374 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>2020/14</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>.384</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>766</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>.1512</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>.7.</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2727/1</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>47/3</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>302/1</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>.156</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>723</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>728/4</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>728/6</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>795/1</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>803</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>971/1</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>.149</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>.154</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1040</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1041</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1043/2</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1044</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1045</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1046</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1118/2</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1207</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2103/7</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>.4047</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>.4046</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>1064/3</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C68" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Latest data: Sun Sep  6 18:01:27 UTC 2026
</commit_message>
<xml_diff>
--- a/docs/particelle_non_trovate.xlsx
+++ b/docs/particelle_non_trovate.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,11 +446,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>506</t>
+          <t>9783/231</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>313</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -459,11 +459,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>824</t>
+          <t>13823</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>313</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4">
@@ -472,11 +472,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>888</t>
+          <t>14724/2</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>313</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5">
@@ -485,11 +485,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>889</t>
+          <t>8974/1</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>313</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6">
@@ -498,11 +498,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>890</t>
+          <t>15380</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>313</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
@@ -511,11 +511,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>891</t>
+          <t>583</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>313</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8">
@@ -524,11 +524,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>897</t>
+          <t>466</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>313</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9">
@@ -537,11 +537,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>898</t>
+          <t>.315</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>313</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10">
@@ -550,11 +550,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>899</t>
+          <t>3298</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>313</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11">
@@ -563,11 +563,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>4119</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>313</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12">
@@ -576,11 +576,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>901</t>
+          <t>4120</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>313</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13">
@@ -589,11 +589,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>9783/231</t>
+          <t>446</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>44</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14">
@@ -602,11 +602,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>13823</t>
+          <t>4523</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>154</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15">
@@ -615,11 +615,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>14724/2</t>
+          <t>2548/13</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>154</v>
+        <v>444</v>
       </c>
     </row>
     <row r="16">
@@ -628,11 +628,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>8974/1</t>
+          <t>1115</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>154</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -641,11 +641,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>15380</t>
+          <t>.451</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>154</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18">
@@ -654,11 +654,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>583</t>
+          <t>274</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>174</v>
+        <v>202</v>
       </c>
     </row>
     <row r="19">
@@ -667,11 +667,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>466</t>
+          <t>1341</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>213</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20">
@@ -680,11 +680,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>.315</t>
+          <t>703</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>282</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21">
@@ -693,11 +693,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3298</t>
+          <t>3597/16</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>257</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -706,11 +706,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>4119</t>
+          <t>3597/18</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>256</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -719,11 +719,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4120</t>
+          <t>3597/22</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>256</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -732,11 +732,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>446</t>
+          <t>3697</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>193</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -745,11 +745,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4523</t>
+          <t>2331/38</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>404</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26">
@@ -758,11 +758,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2548/13</t>
+          <t>2068/43</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>444</v>
+        <v>310</v>
       </c>
     </row>
     <row r="27">
@@ -771,11 +771,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1115</t>
+          <t>2822/12</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7</v>
+        <v>310</v>
       </c>
     </row>
     <row r="28">
@@ -784,11 +784,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>.451</t>
+          <t>2822/16</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>88</v>
+        <v>310</v>
       </c>
     </row>
     <row r="29">
@@ -797,11 +797,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>2020/14</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>202</v>
+        <v>310</v>
       </c>
     </row>
     <row r="30">
@@ -810,11 +810,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1341</t>
+          <t>.384</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31">
@@ -823,11 +823,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>766</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>61</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32">
@@ -836,11 +836,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>3597/16</t>
+          <t>.1512</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33">
@@ -849,11 +849,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>3597/18</t>
+          <t>.7.</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34">
@@ -862,11 +862,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>3597/22</t>
+          <t>2727/1</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35">
@@ -875,11 +875,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>3697</t>
+          <t>47/3</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>9</v>
+        <v>277</v>
       </c>
     </row>
     <row r="36">
@@ -888,11 +888,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2331/38</t>
+          <t>302/1</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>258</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37">
@@ -901,11 +901,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2068/43</t>
+          <t>2103/7</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>310</v>
+        <v>394</v>
       </c>
     </row>
     <row r="38">
@@ -914,11 +914,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2822/12</t>
+          <t>.4047</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="39">
@@ -927,11 +927,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2822/16</t>
+          <t>.4046</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="40">
@@ -940,374 +940,10 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2020/14</t>
+          <t>1064/3</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>.384</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>766</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>.1512</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>.7.</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2727/1</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>47/3</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>302/1</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>.156</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>723</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>728/4</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>728/6</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>795/1</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>803</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>971/1</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>.149</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>.154</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>1040</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>1041</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>1043/2</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>58</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>1044</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>59</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>1045</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>60</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>1046</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>61</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>1118/2</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>62</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>1207</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>63</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>2103/7</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>64</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>.4047</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>65</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>.4046</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>66</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>1064/3</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
         <v>248</v>
       </c>
     </row>

</xml_diff>